<commit_message>
particiones K=2...3 Qnodes y GeoMip
</commit_message>
<xml_diff>
--- a/GeoMIP/results/resultados_Geometric.xlsx
+++ b/GeoMIP/results/resultados_Geometric.xlsx
@@ -17,16 +17,13 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="2">
+  <fonts count="1">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
       <color theme="1"/>
       <sz val="11"/>
       <scheme val="minor"/>
-    </font>
-    <font>
-      <b val="1"/>
     </font>
   </fonts>
   <fills count="2">
@@ -37,7 +34,7 @@
       <patternFill patternType="gray125"/>
     </fill>
   </fills>
-  <borders count="2">
+  <borders count="1">
     <border>
       <left/>
       <right/>
@@ -45,21 +42,12 @@
       <bottom/>
       <diagonal/>
     </border>
-    <border>
-      <left style="thin"/>
-      <right style="thin"/>
-      <top style="thin"/>
-      <bottom style="thin"/>
-    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="top"/>
-    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -429,32 +417,32 @@
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
-      <c r="A1" s="1" t="inlineStr">
+      <c r="A1" t="inlineStr">
         <is>
           <t>Iteración</t>
         </is>
       </c>
-      <c r="B1" s="1" t="inlineStr">
+      <c r="B1" t="inlineStr">
         <is>
           <t>Alcance</t>
         </is>
       </c>
-      <c r="C1" s="1" t="inlineStr">
+      <c r="C1" t="inlineStr">
         <is>
           <t>Mecanismo</t>
         </is>
       </c>
-      <c r="D1" s="1" t="inlineStr">
+      <c r="D1" t="inlineStr">
         <is>
           <t>Partición</t>
         </is>
       </c>
-      <c r="E1" s="1" t="inlineStr">
+      <c r="E1" t="inlineStr">
         <is>
           <t>Pérdida</t>
         </is>
       </c>
-      <c r="F1" s="1" t="inlineStr">
+      <c r="F1" t="inlineStr">
         <is>
           <t>Tiempo de ejecución (s)</t>
         </is>
@@ -466,28 +454,28 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>111111111111111</t>
+          <t>111111111100000</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>111111111111111</t>
+          <t>111111111100000</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>| A,B,C,D,E,F,G,H,I,J,K,L,M,N,O || ∅ |
-|  b,c,d,e,f,g,h,i,j,k,l,m,n,o  || a |</t>
+          <t>|  A,B,C,D,E,F,H,I,J  || G |
+| a,b,c,d,e,f,g,h,i,j || ∅ |</t>
         </is>
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>0,0</t>
+          <t>0,00026786327</t>
         </is>
       </c>
       <c r="F2" t="inlineStr">
         <is>
-          <t>5,352838039398193</t>
+          <t>0,1597752571105957</t>
         </is>
       </c>
     </row>
@@ -497,28 +485,28 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>111111111111111</t>
+          <t>111111111100000</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>111111111111111</t>
+          <t>111111111000000</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>| A,B,C,D,E,F,G,H,I,J,K,L,M,N,O || ∅ |
-|  b,c,d,e,f,g,h,i,j,k,l,m,n,o  || a |</t>
+          <t>| A,B,C,D,E,G,H,I,J || F |
+| a,b,c,d,e,f,g,h,i || ∅ |</t>
         </is>
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>0,0</t>
+          <t>0,0016031265</t>
         </is>
       </c>
       <c r="F3" t="inlineStr">
         <is>
-          <t>4,6584813594818115</t>
+          <t>0,08880996704101562</t>
         </is>
       </c>
     </row>
@@ -528,28 +516,28 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>111111111111111</t>
+          <t>111111111100000</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>011111111111111</t>
+          <t>011111111100000</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>| A,B,C,D,E,F,G,H,I,J,K,L,M,N,O || ∅ |
-|   c,d,e,f,g,h,i,j,k,l,m,n,o   || b |</t>
+          <t>| A,B,C,E,F,G,H,I,J || D |
+| b,c,d,e,f,g,h,i,j || ∅ |</t>
         </is>
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>0,0</t>
+          <t>0,0002501011</t>
         </is>
       </c>
       <c r="F4" t="inlineStr">
         <is>
-          <t>2,1104185581207275</t>
+          <t>0,1039581298828125</t>
         </is>
       </c>
     </row>
@@ -559,28 +547,28 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>111111111111111</t>
+          <t>111111111100000</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>011111111111111</t>
+          <t>011111111000000</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>| A,B,C,D,E,F,G,H,I,J,K,L,M,N,O || ∅ |
-|   c,d,e,f,g,h,i,j,k,l,m,n,o   || b |</t>
+          <t>| A,B,C,D,E,F,G,H,J || I |
+|  b,c,d,e,f,g,h,i  || ∅ |</t>
         </is>
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>0,0</t>
+          <t>0,0021489859</t>
         </is>
       </c>
       <c r="F5" t="inlineStr">
         <is>
-          <t>2,262632131576538</t>
+          <t>0,06783342361450195</t>
         </is>
       </c>
     </row>
@@ -590,28 +578,28 @@
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>111111111111111</t>
+          <t>111111111100000</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>101010101010101</t>
+          <t>101010101000000</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>| A,B,C,D,E,F,G,H,I,J,K,M,N,O || L |
-|       a,c,e,g,i,k,m,o       || ∅ |</t>
+          <t>| A,B,C,D,E,F,G,H,J || I |
+|     a,c,e,g,i     || ∅ |</t>
         </is>
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>0,0041897893</t>
+          <t>0,00075376034</t>
         </is>
       </c>
       <c r="F6" t="inlineStr">
         <is>
-          <t>0,06342649459838867</t>
+          <t>0,03400826454162598</t>
         </is>
       </c>
     </row>
@@ -621,28 +609,28 @@
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>111111111111111</t>
+          <t>111111111100000</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>010101010101010</t>
+          <t>010101010100000</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>| A,B,C,D,E,F,H,I,J,K,L,M,N,O || G |
-|        b,d,f,h,j,l,n        || ∅ |</t>
+          <t>| A,B,D,E,F,G,H,I,J || C |
+|     b,d,f,h,j     || ∅ |</t>
         </is>
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t>0,0070973635</t>
+          <t>0,00035369396</t>
         </is>
       </c>
       <c r="F7" t="inlineStr">
         <is>
-          <t>0,049510955810546875</t>
+          <t>0,035151004791259766</t>
         </is>
       </c>
     </row>
@@ -652,28 +640,28 @@
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>111111111111111</t>
+          <t>111111111100000</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>110110110110110</t>
+          <t>110110110100000</t>
         </is>
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>| A,B,C,D,E,F,G,H,I,J,K,L,M,N || O |
-|     a,b,d,e,g,h,j,k,m,n     || ∅ |</t>
+          <t>| B,C,D,E,F,G,H,I,J || A |
+|   a,b,d,e,g,h,j   || ∅ |</t>
         </is>
       </c>
       <c r="E8" t="inlineStr">
         <is>
-          <t>4,7147274e-05</t>
+          <t>0,0013819933</t>
         </is>
       </c>
       <c r="F8" t="inlineStr">
         <is>
-          <t>0,13635802268981934</t>
+          <t>0,05988192558288574</t>
         </is>
       </c>
     </row>
@@ -683,28 +671,28 @@
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>111111111111111</t>
+          <t>111111111000000</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>111111111111111</t>
+          <t>111111111100000</t>
         </is>
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>| A,B,C,D,E,F,G,H,I,J,K,L,M,N,O || ∅ |
-|  b,c,d,e,f,g,h,i,j,k,l,m,n,o  || a |</t>
+          <t>|   A,B,C,D,E,F,H,I   || G |
+| a,b,c,d,e,f,g,h,i,j || ∅ |</t>
         </is>
       </c>
       <c r="E9" t="inlineStr">
         <is>
-          <t>0,0</t>
+          <t>0,00026786327</t>
         </is>
       </c>
       <c r="F9" t="inlineStr">
         <is>
-          <t>4,714722633361816</t>
+          <t>0,20430946350097656</t>
         </is>
       </c>
     </row>
@@ -714,28 +702,28 @@
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>111111111111111</t>
+          <t>111111111000000</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>111111111111111</t>
+          <t>111111111000000</t>
         </is>
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>| A,B,C,D,E,F,G,H,I,J,K,L,M,N,O || ∅ |
-|  b,c,d,e,f,g,h,i,j,k,l,m,n,o  || a |</t>
+          <t>|  A,B,C,D,E,G,H,I  || F |
+| a,b,c,d,e,f,g,h,i || ∅ |</t>
         </is>
       </c>
       <c r="E10" t="inlineStr">
         <is>
-          <t>0,0</t>
+          <t>0,0016031265</t>
         </is>
       </c>
       <c r="F10" t="inlineStr">
         <is>
-          <t>4,803154230117798</t>
+          <t>0,11518478393554688</t>
         </is>
       </c>
     </row>
@@ -745,28 +733,28 @@
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>111111111111111</t>
+          <t>111111111000000</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>011111111111111</t>
+          <t>011111111100000</t>
         </is>
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>| A,B,C,D,E,F,G,H,I,J,K,L,M,N,O || ∅ |
-|   c,d,e,f,g,h,i,j,k,l,m,n,o   || b |</t>
+          <t>|  A,B,C,E,F,G,H,I  || D |
+| b,c,d,e,f,g,h,i,j || ∅ |</t>
         </is>
       </c>
       <c r="E11" t="inlineStr">
         <is>
-          <t>0,0</t>
+          <t>0,0002501011</t>
         </is>
       </c>
       <c r="F11" t="inlineStr">
         <is>
-          <t>2,2647907733917236</t>
+          <t>0,07639789581298828</t>
         </is>
       </c>
     </row>
@@ -776,28 +764,28 @@
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>111111111111111</t>
+          <t>111111111000000</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>011111111111111</t>
+          <t>011111111000000</t>
         </is>
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>| A,B,C,D,E,F,G,H,I,J,K,L,M,N,O || ∅ |
-|   c,d,e,f,g,h,i,j,k,l,m,n,o   || b |</t>
+          <t>| A,B,C,D,E,F,G,H || I |
+| b,c,d,e,f,g,h,i || ∅ |</t>
         </is>
       </c>
       <c r="E12" t="inlineStr">
         <is>
-          <t>0,0</t>
+          <t>0,0021489859</t>
         </is>
       </c>
       <c r="F12" t="inlineStr">
         <is>
-          <t>2,1691153049468994</t>
+          <t>0,07098245620727539</t>
         </is>
       </c>
     </row>
@@ -807,28 +795,28 @@
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>111111111111111</t>
+          <t>111111111000000</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>101010101010101</t>
+          <t>101010101000000</t>
         </is>
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t>| A,B,C,D,E,F,G,H,I,J,K,M,N,O || L |
-|       a,c,e,g,i,k,m,o       || ∅ |</t>
+          <t>| A,B,C,D,E,F,G,H || I |
+|    a,c,e,g,i    || ∅ |</t>
         </is>
       </c>
       <c r="E13" t="inlineStr">
         <is>
-          <t>0,0041897893</t>
+          <t>0,00075376034</t>
         </is>
       </c>
       <c r="F13" t="inlineStr">
         <is>
-          <t>0,05904340744018555</t>
+          <t>0,059220314025878906</t>
         </is>
       </c>
     </row>
@@ -838,28 +826,28 @@
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>111111111111111</t>
+          <t>111111111000000</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>010101010101010</t>
+          <t>010101010100000</t>
         </is>
       </c>
       <c r="D14" t="inlineStr">
         <is>
-          <t>| A,B,C,D,E,F,H,I,J,K,L,M,N,O || G |
-|        b,d,f,h,j,l,n        || ∅ |</t>
+          <t>| A,B,D,E,F,G,H,I || C |
+|    b,d,f,h,j    || ∅ |</t>
         </is>
       </c>
       <c r="E14" t="inlineStr">
         <is>
-          <t>0,0070973635</t>
+          <t>0,00035369396</t>
         </is>
       </c>
       <c r="F14" t="inlineStr">
         <is>
-          <t>0,0414583683013916</t>
+          <t>0,04262113571166992</t>
         </is>
       </c>
     </row>
@@ -869,28 +857,28 @@
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>111111111111111</t>
+          <t>111111111000000</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>110110110110110</t>
+          <t>110110110100000</t>
         </is>
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t>| A,B,C,D,E,F,G,H,I,J,K,L,M,N || O |
-|     a,b,d,e,g,h,j,k,m,n     || ∅ |</t>
+          <t>| B,C,D,E,F,G,H,I || A |
+|  a,b,d,e,g,h,j  || ∅ |</t>
         </is>
       </c>
       <c r="E15" t="inlineStr">
         <is>
-          <t>4,7147274e-05</t>
+          <t>0,0013819933</t>
         </is>
       </c>
       <c r="F15" t="inlineStr">
         <is>
-          <t>0,14406967163085938</t>
+          <t>0,05911660194396973</t>
         </is>
       </c>
     </row>
@@ -900,28 +888,28 @@
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>011111111111111</t>
+          <t>011111111100000</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>111111111111111</t>
+          <t>111111111100000</t>
         </is>
       </c>
       <c r="D16" t="inlineStr">
         <is>
-          <t>| B,C,D,E,F,G,H,I,J,K,L,M,N,O || ∅ |
-| b,c,d,e,f,g,h,i,j,k,l,m,n,o || a |</t>
+          <t>|   B,C,D,E,F,H,I,J   || G |
+| a,b,c,d,e,f,g,h,i,j || ∅ |</t>
         </is>
       </c>
       <c r="E16" t="inlineStr">
         <is>
-          <t>0,0</t>
+          <t>0,00026786327</t>
         </is>
       </c>
       <c r="F16" t="inlineStr">
         <is>
-          <t>4,932002305984497</t>
+          <t>0,22381138801574707</t>
         </is>
       </c>
     </row>
@@ -931,28 +919,28 @@
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>011111111111111</t>
+          <t>011111111100000</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>111111111111111</t>
+          <t>111111111000000</t>
         </is>
       </c>
       <c r="D17" t="inlineStr">
         <is>
-          <t>| B,C,D,E,F,G,H,I,J,K,L,M,N,O || ∅ |
-| b,c,d,e,f,g,h,i,j,k,l,m,n,o || a |</t>
+          <t>|  B,C,D,E,G,H,I,J  || F |
+| a,b,c,d,e,f,g,h,i || ∅ |</t>
         </is>
       </c>
       <c r="E17" t="inlineStr">
         <is>
-          <t>0,0</t>
+          <t>0,0016031265</t>
         </is>
       </c>
       <c r="F17" t="inlineStr">
         <is>
-          <t>5,199156284332275</t>
+          <t>0,1109769344329834</t>
         </is>
       </c>
     </row>
@@ -962,28 +950,28 @@
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>011111111111111</t>
+          <t>011111111100000</t>
         </is>
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>011111111111111</t>
+          <t>011111111100000</t>
         </is>
       </c>
       <c r="D18" t="inlineStr">
         <is>
-          <t>| B,C,D,E,F,G,H,I,J,K,L,M,N,O || ∅ |
-|  c,d,e,f,g,h,i,j,k,l,m,n,o  || b |</t>
+          <t>|  B,C,E,F,G,H,I,J  || D |
+| b,c,d,e,f,g,h,i,j || ∅ |</t>
         </is>
       </c>
       <c r="E18" t="inlineStr">
         <is>
-          <t>0,0</t>
+          <t>0,0002501011</t>
         </is>
       </c>
       <c r="F18" t="inlineStr">
         <is>
-          <t>2,081904649734497</t>
+          <t>0,11030697822570801</t>
         </is>
       </c>
     </row>
@@ -993,28 +981,28 @@
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>011111111111111</t>
+          <t>011111111100000</t>
         </is>
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>011111111111111</t>
+          <t>011111111000000</t>
         </is>
       </c>
       <c r="D19" t="inlineStr">
         <is>
-          <t>| B,C,D,E,F,G,H,I,J,K,L,M,N,O || ∅ |
-|  c,d,e,f,g,h,i,j,k,l,m,n,o  || b |</t>
+          <t>| B,C,D,E,F,G,H,J || I |
+| b,c,d,e,f,g,h,i || ∅ |</t>
         </is>
       </c>
       <c r="E19" t="inlineStr">
         <is>
-          <t>0,0</t>
+          <t>0,0021489859</t>
         </is>
       </c>
       <c r="F19" t="inlineStr">
         <is>
-          <t>2,1407582759857178</t>
+          <t>0,07039618492126465</t>
         </is>
       </c>
     </row>
@@ -1024,28 +1012,28 @@
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>011111111111111</t>
+          <t>011111111100000</t>
         </is>
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>101010101010101</t>
+          <t>101010101000000</t>
         </is>
       </c>
       <c r="D20" t="inlineStr">
         <is>
-          <t>| B,C,D,E,F,G,H,I,J,K,M,N,O || L |
-|      a,c,e,g,i,k,m,o      || ∅ |</t>
+          <t>| B,C,D,E,F,G,H,J || I |
+|    a,c,e,g,i    || ∅ |</t>
         </is>
       </c>
       <c r="E20" t="inlineStr">
         <is>
-          <t>0,0041897893</t>
+          <t>0,00075376034</t>
         </is>
       </c>
       <c r="F20" t="inlineStr">
         <is>
-          <t>0,10186362266540527</t>
+          <t>0,03347420692443848</t>
         </is>
       </c>
     </row>
@@ -1055,28 +1043,28 @@
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>011111111111111</t>
+          <t>011111111100000</t>
         </is>
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>010101010101010</t>
+          <t>010101010100000</t>
         </is>
       </c>
       <c r="D21" t="inlineStr">
         <is>
-          <t>| B,C,D,E,F,H,I,J,K,L,M,N,O || G |
-|       b,d,f,h,j,l,n       || ∅ |</t>
+          <t>| B,D,E,F,G,H,I,J || C |
+|    b,d,f,h,j    || ∅ |</t>
         </is>
       </c>
       <c r="E21" t="inlineStr">
         <is>
-          <t>0,0070973635</t>
+          <t>0,00035369396</t>
         </is>
       </c>
       <c r="F21" t="inlineStr">
         <is>
-          <t>0,04098963737487793</t>
+          <t>0,0362248420715332</t>
         </is>
       </c>
     </row>
@@ -1086,28 +1074,28 @@
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>011111111111111</t>
+          <t>011111111100000</t>
         </is>
       </c>
       <c r="C22" t="inlineStr">
         <is>
-          <t>110110110110110</t>
+          <t>110110110100000</t>
         </is>
       </c>
       <c r="D22" t="inlineStr">
         <is>
-          <t>| B,C,D,E,F,G,H,I,J,K,L,M,N || O |
-|    a,b,d,e,g,h,j,k,m,n    || ∅ |</t>
+          <t>| B,C,E,F,G,H,I,J || D |
+|  a,b,d,e,g,h,j  || ∅ |</t>
         </is>
       </c>
       <c r="E22" t="inlineStr">
         <is>
-          <t>4,7147274e-05</t>
+          <t>0,0015337467</t>
         </is>
       </c>
       <c r="F22" t="inlineStr">
         <is>
-          <t>0,12781715393066406</t>
+          <t>0,04820561408996582</t>
         </is>
       </c>
     </row>
@@ -1117,28 +1105,28 @@
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>011111111111111</t>
+          <t>011111111000000</t>
         </is>
       </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t>111111111111111</t>
+          <t>111111111100000</t>
         </is>
       </c>
       <c r="D23" t="inlineStr">
         <is>
-          <t>| B,C,D,E,F,G,H,I,J,K,L,M,N,O || ∅ |
-| b,c,d,e,f,g,h,i,j,k,l,m,n,o || a |</t>
+          <t>|    B,C,D,E,F,H,I    || G |
+| a,b,c,d,e,f,g,h,i,j || ∅ |</t>
         </is>
       </c>
       <c r="E23" t="inlineStr">
         <is>
-          <t>0,0</t>
+          <t>0,00026786327</t>
         </is>
       </c>
       <c r="F23" t="inlineStr">
         <is>
-          <t>4,814034461975098</t>
+          <t>0,13620734214782715</t>
         </is>
       </c>
     </row>
@@ -1148,28 +1136,28 @@
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>011111111111111</t>
+          <t>011111111000000</t>
         </is>
       </c>
       <c r="C24" t="inlineStr">
         <is>
-          <t>111111111111111</t>
+          <t>111111111000000</t>
         </is>
       </c>
       <c r="D24" t="inlineStr">
         <is>
-          <t>| B,C,D,E,F,G,H,I,J,K,L,M,N,O || ∅ |
-| b,c,d,e,f,g,h,i,j,k,l,m,n,o || a |</t>
+          <t>|   B,C,D,E,G,H,I   || F |
+| a,b,c,d,e,f,g,h,i || ∅ |</t>
         </is>
       </c>
       <c r="E24" t="inlineStr">
         <is>
-          <t>0,0</t>
+          <t>0,0016031265</t>
         </is>
       </c>
       <c r="F24" t="inlineStr">
         <is>
-          <t>4,430880308151245</t>
+          <t>0,10329437255859375</t>
         </is>
       </c>
     </row>
@@ -1179,28 +1167,28 @@
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>011111111111111</t>
+          <t>011111111000000</t>
         </is>
       </c>
       <c r="C25" t="inlineStr">
         <is>
-          <t>011111111111111</t>
+          <t>011111111100000</t>
         </is>
       </c>
       <c r="D25" t="inlineStr">
         <is>
-          <t>| B,C,D,E,F,G,H,I,J,K,L,M,N,O || ∅ |
-|  c,d,e,f,g,h,i,j,k,l,m,n,o  || b |</t>
+          <t>|   B,C,E,F,G,H,I   || D |
+| b,c,d,e,f,g,h,i,j || ∅ |</t>
         </is>
       </c>
       <c r="E25" t="inlineStr">
         <is>
-          <t>0,0</t>
+          <t>0,0002501011</t>
         </is>
       </c>
       <c r="F25" t="inlineStr">
         <is>
-          <t>2,1023313999176025</t>
+          <t>0,09270572662353516</t>
         </is>
       </c>
     </row>
@@ -1210,28 +1198,28 @@
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>011111111111111</t>
+          <t>011111111000000</t>
         </is>
       </c>
       <c r="C26" t="inlineStr">
         <is>
-          <t>011111111111111</t>
+          <t>011111111000000</t>
         </is>
       </c>
       <c r="D26" t="inlineStr">
         <is>
-          <t>| B,C,D,E,F,G,H,I,J,K,L,M,N,O || ∅ |
-|  c,d,e,f,g,h,i,j,k,l,m,n,o  || b |</t>
+          <t>|  B,C,D,E,F,G,H  || I |
+| b,c,d,e,f,g,h,i || ∅ |</t>
         </is>
       </c>
       <c r="E26" t="inlineStr">
         <is>
-          <t>0,0</t>
+          <t>0,0021489859</t>
         </is>
       </c>
       <c r="F26" t="inlineStr">
         <is>
-          <t>2,0792903900146484</t>
+          <t>0,07706165313720703</t>
         </is>
       </c>
     </row>
@@ -1241,28 +1229,28 @@
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>011111111111111</t>
+          <t>011111111000000</t>
         </is>
       </c>
       <c r="C27" t="inlineStr">
         <is>
-          <t>101010101010101</t>
+          <t>101010101000000</t>
         </is>
       </c>
       <c r="D27" t="inlineStr">
         <is>
-          <t>| B,C,D,E,F,G,H,I,J,K,M,N,O || L |
-|      a,c,e,g,i,k,m,o      || ∅ |</t>
+          <t>| B,C,D,E,F,G,H || I |
+|   a,c,e,g,i   || ∅ |</t>
         </is>
       </c>
       <c r="E27" t="inlineStr">
         <is>
-          <t>0,0041897893</t>
+          <t>0,00075376034</t>
         </is>
       </c>
       <c r="F27" t="inlineStr">
         <is>
-          <t>0,05192065238952637</t>
+          <t>0,03278660774230957</t>
         </is>
       </c>
     </row>
@@ -1272,28 +1260,28 @@
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>011111111111111</t>
+          <t>011111111000000</t>
         </is>
       </c>
       <c r="C28" t="inlineStr">
         <is>
-          <t>010101010101010</t>
+          <t>010101010100000</t>
         </is>
       </c>
       <c r="D28" t="inlineStr">
         <is>
-          <t>| B,C,D,E,F,H,I,J,K,L,M,N,O || G |
-|       b,d,f,h,j,l,n       || ∅ |</t>
+          <t>| B,D,E,F,G,H,I || C |
+|   b,d,f,h,j   || ∅ |</t>
         </is>
       </c>
       <c r="E28" t="inlineStr">
         <is>
-          <t>0,0070973635</t>
+          <t>0,00035369396</t>
         </is>
       </c>
       <c r="F28" t="inlineStr">
         <is>
-          <t>0,042236328125</t>
+          <t>0,027979373931884766</t>
         </is>
       </c>
     </row>
@@ -1303,28 +1291,28 @@
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>011111111111111</t>
+          <t>011111111000000</t>
         </is>
       </c>
       <c r="C29" t="inlineStr">
         <is>
-          <t>110110110110110</t>
+          <t>110110110100000</t>
         </is>
       </c>
       <c r="D29" t="inlineStr">
         <is>
-          <t>| B,C,D,E,F,G,H,I,J,K,L,M,N || O |
-|    a,b,d,e,g,h,j,k,m,n    || ∅ |</t>
+          <t>| B,C,E,F,G,H,I || D |
+| a,b,d,e,g,h,j || ∅ |</t>
         </is>
       </c>
       <c r="E29" t="inlineStr">
         <is>
-          <t>4,7147274e-05</t>
+          <t>0,0015337467</t>
         </is>
       </c>
       <c r="F29" t="inlineStr">
         <is>
-          <t>0,12509489059448242</t>
+          <t>0,044114112854003906</t>
         </is>
       </c>
     </row>
@@ -1334,28 +1322,28 @@
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t>101010101010101</t>
+          <t>101010101000000</t>
         </is>
       </c>
       <c r="C30" t="inlineStr">
         <is>
-          <t>111111111111111</t>
+          <t>111111111100000</t>
         </is>
       </c>
       <c r="D30" t="inlineStr">
         <is>
-          <t>|       A,C,E,G,I,K,M,O       || ∅ |
-| b,c,d,e,f,g,h,i,j,k,l,m,n,o || a |</t>
+          <t>|       A,C,E,I       || G |
+| a,b,c,d,e,f,g,h,i,j || ∅ |</t>
         </is>
       </c>
       <c r="E30" t="inlineStr">
         <is>
-          <t>0,0</t>
+          <t>0,00026786327</t>
         </is>
       </c>
       <c r="F30" t="inlineStr">
         <is>
-          <t>3,4753942489624023</t>
+          <t>0,17999792098999023</t>
         </is>
       </c>
     </row>
@@ -1365,28 +1353,28 @@
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>101010101010101</t>
+          <t>101010101000000</t>
         </is>
       </c>
       <c r="C31" t="inlineStr">
         <is>
-          <t>111111111111111</t>
+          <t>111111111000000</t>
         </is>
       </c>
       <c r="D31" t="inlineStr">
         <is>
-          <t>|       A,C,E,G,I,K,M,O       || ∅ |
-| b,c,d,e,f,g,h,i,j,k,l,m,n,o || a |</t>
+          <t>|      A,C,E,G      || I |
+| a,b,c,d,e,f,g,h,i || ∅ |</t>
         </is>
       </c>
       <c r="E31" t="inlineStr">
         <is>
-          <t>0,0</t>
+          <t>0,0031766295</t>
         </is>
       </c>
       <c r="F31" t="inlineStr">
         <is>
-          <t>3,5138235092163086</t>
+          <t>0,07726883888244629</t>
         </is>
       </c>
     </row>
@@ -1396,28 +1384,28 @@
       </c>
       <c r="B32" t="inlineStr">
         <is>
-          <t>101010101010101</t>
+          <t>101010101000000</t>
         </is>
       </c>
       <c r="C32" t="inlineStr">
         <is>
-          <t>011111111111111</t>
+          <t>011111111100000</t>
         </is>
       </c>
       <c r="D32" t="inlineStr">
         <is>
-          <t>|      A,C,E,G,I,K,M,O      || ∅ |
-| c,d,e,f,g,h,i,j,k,l,m,n,o || b |</t>
+          <t>|      A,C,G,I      || E |
+| b,c,d,e,f,g,h,i,j || ∅ |</t>
         </is>
       </c>
       <c r="E32" t="inlineStr">
         <is>
-          <t>0,0</t>
+          <t>0,0010385513</t>
         </is>
       </c>
       <c r="F32" t="inlineStr">
         <is>
-          <t>1,575566291809082</t>
+          <t>0,07395315170288086</t>
         </is>
       </c>
     </row>
@@ -1427,28 +1415,28 @@
       </c>
       <c r="B33" t="inlineStr">
         <is>
-          <t>101010101010101</t>
+          <t>101010101000000</t>
         </is>
       </c>
       <c r="C33" t="inlineStr">
         <is>
-          <t>011111111111111</t>
+          <t>011111111000000</t>
         </is>
       </c>
       <c r="D33" t="inlineStr">
         <is>
-          <t>|      A,C,E,G,I,K,M,O      || ∅ |
-| c,d,e,f,g,h,i,j,k,l,m,n,o || b |</t>
+          <t>|     A,C,E,G     || I |
+| b,c,d,e,f,g,h,i || ∅ |</t>
         </is>
       </c>
       <c r="E33" t="inlineStr">
         <is>
-          <t>0,0</t>
+          <t>0,0021489859</t>
         </is>
       </c>
       <c r="F33" t="inlineStr">
         <is>
-          <t>1,625032663345337</t>
+          <t>0,0422670841217041</t>
         </is>
       </c>
     </row>
@@ -1458,28 +1446,28 @@
       </c>
       <c r="B34" t="inlineStr">
         <is>
-          <t>101010101010101</t>
+          <t>101010101000000</t>
         </is>
       </c>
       <c r="C34" t="inlineStr">
         <is>
-          <t>101010101010101</t>
+          <t>101010101000000</t>
         </is>
       </c>
       <c r="D34" t="inlineStr">
         <is>
-          <t>|  A,C,G,I,K,M,O  || E |
-| a,c,e,g,i,k,m,o || ∅ |</t>
+          <t>|  A,C,E,G  || I |
+| a,c,e,g,i || ∅ |</t>
         </is>
       </c>
       <c r="E34" t="inlineStr">
         <is>
-          <t>0,0043781996</t>
+          <t>0,00075376034</t>
         </is>
       </c>
       <c r="F34" t="inlineStr">
         <is>
-          <t>0,033789873123168945</t>
+          <t>0,018315792083740234</t>
         </is>
       </c>
     </row>
@@ -1489,28 +1477,28 @@
       </c>
       <c r="B35" t="inlineStr">
         <is>
-          <t>101010101010101</t>
+          <t>101010101000000</t>
         </is>
       </c>
       <c r="C35" t="inlineStr">
         <is>
-          <t>010101010101010</t>
+          <t>010101010100000</t>
         </is>
       </c>
       <c r="D35" t="inlineStr">
         <is>
-          <t>| A,C,E,I,K,M,O || G |
-| b,d,f,h,j,l,n || ∅ |</t>
+          <t>|  A,E,G,I  || C |
+| b,d,f,h,j || ∅ |</t>
         </is>
       </c>
       <c r="E35" t="inlineStr">
         <is>
-          <t>0,0070973635</t>
+          <t>0,00035369396</t>
         </is>
       </c>
       <c r="F35" t="inlineStr">
         <is>
-          <t>0,018452882766723633</t>
+          <t>0,015765666961669922</t>
         </is>
       </c>
     </row>
@@ -1520,28 +1508,28 @@
       </c>
       <c r="B36" t="inlineStr">
         <is>
-          <t>101010101010101</t>
+          <t>101010101000000</t>
         </is>
       </c>
       <c r="C36" t="inlineStr">
         <is>
-          <t>110110110110110</t>
+          <t>110110110100000</t>
         </is>
       </c>
       <c r="D36" t="inlineStr">
         <is>
-          <t>|    A,C,E,G,I,K,M    || O |
-| a,b,d,e,g,h,j,k,m,n || ∅ |</t>
+          <t>|    C,E,G,I    || A |
+| a,b,d,e,g,h,j || ∅ |</t>
         </is>
       </c>
       <c r="E36" t="inlineStr">
         <is>
-          <t>4,7147274e-05</t>
+          <t>0,0013819933</t>
         </is>
       </c>
       <c r="F36" t="inlineStr">
         <is>
-          <t>0,09089827537536621</t>
+          <t>0,024560928344726562</t>
         </is>
       </c>
     </row>
@@ -1551,28 +1539,28 @@
       </c>
       <c r="B37" t="inlineStr">
         <is>
-          <t>010101010101010</t>
+          <t>010101010100000</t>
         </is>
       </c>
       <c r="C37" t="inlineStr">
         <is>
-          <t>111111111111111</t>
+          <t>111111111100000</t>
         </is>
       </c>
       <c r="D37" t="inlineStr">
         <is>
-          <t>|        B,D,F,H,J,L,N        || ∅ |
-| b,c,d,e,f,g,h,i,j,k,l,m,n,o || a |</t>
+          <t>|       B,D,F,H       || J |
+| a,b,c,d,e,f,g,h,i,j || ∅ |</t>
         </is>
       </c>
       <c r="E37" t="inlineStr">
         <is>
-          <t>0,0</t>
+          <t>0,0007697344</t>
         </is>
       </c>
       <c r="F37" t="inlineStr">
         <is>
-          <t>3,3107752799987793</t>
+          <t>0,16044330596923828</t>
         </is>
       </c>
     </row>
@@ -1582,28 +1570,28 @@
       </c>
       <c r="B38" t="inlineStr">
         <is>
-          <t>010101010101010</t>
+          <t>010101010100000</t>
         </is>
       </c>
       <c r="C38" t="inlineStr">
         <is>
-          <t>111111111111111</t>
+          <t>111111111000000</t>
         </is>
       </c>
       <c r="D38" t="inlineStr">
         <is>
-          <t>|        B,D,F,H,J,L,N        || ∅ |
-| b,c,d,e,f,g,h,i,j,k,l,m,n,o || a |</t>
+          <t>|      B,D,H,J      || F |
+| a,b,c,d,e,f,g,h,i || ∅ |</t>
         </is>
       </c>
       <c r="E38" t="inlineStr">
         <is>
-          <t>0,0</t>
+          <t>0,0016031265</t>
         </is>
       </c>
       <c r="F38" t="inlineStr">
         <is>
-          <t>3,2863988876342773</t>
+          <t>0,08644986152648926</t>
         </is>
       </c>
     </row>
@@ -1613,28 +1601,28 @@
       </c>
       <c r="B39" t="inlineStr">
         <is>
-          <t>010101010101010</t>
+          <t>010101010100000</t>
         </is>
       </c>
       <c r="C39" t="inlineStr">
         <is>
-          <t>011111111111111</t>
+          <t>011111111100000</t>
         </is>
       </c>
       <c r="D39" t="inlineStr">
         <is>
-          <t>|       B,D,F,H,J,L,N       || ∅ |
-| c,d,e,f,g,h,i,j,k,l,m,n,o || b |</t>
+          <t>|      B,F,H,J      || D |
+| b,c,d,e,f,g,h,i,j || ∅ |</t>
         </is>
       </c>
       <c r="E39" t="inlineStr">
         <is>
-          <t>0,0</t>
+          <t>0,0002501011</t>
         </is>
       </c>
       <c r="F39" t="inlineStr">
         <is>
-          <t>1,5640175342559814</t>
+          <t>0,08224272727966309</t>
         </is>
       </c>
     </row>
@@ -1644,28 +1632,28 @@
       </c>
       <c r="B40" t="inlineStr">
         <is>
-          <t>010101010101010</t>
+          <t>010101010100000</t>
         </is>
       </c>
       <c r="C40" t="inlineStr">
         <is>
-          <t>011111111111111</t>
+          <t>011111111000000</t>
         </is>
       </c>
       <c r="D40" t="inlineStr">
         <is>
-          <t>|       B,D,F,H,J,L,N       || ∅ |
-| c,d,e,f,g,h,i,j,k,l,m,n,o || b |</t>
+          <t>|     B,D,F,H     || J |
+| b,c,d,e,f,g,h,i || ∅ |</t>
         </is>
       </c>
       <c r="E40" t="inlineStr">
         <is>
-          <t>0,0</t>
+          <t>0,0030118823</t>
         </is>
       </c>
       <c r="F40" t="inlineStr">
         <is>
-          <t>1,5321049690246582</t>
+          <t>0,04714345932006836</t>
         </is>
       </c>
     </row>
@@ -1675,28 +1663,28 @@
       </c>
       <c r="B41" t="inlineStr">
         <is>
-          <t>010101010101010</t>
+          <t>010101010100000</t>
         </is>
       </c>
       <c r="C41" t="inlineStr">
         <is>
-          <t>101010101010101</t>
+          <t>101010101000000</t>
         </is>
       </c>
       <c r="D41" t="inlineStr">
         <is>
-          <t>|   B,D,F,H,J,N   || L |
-| a,c,e,g,i,k,m,o || ∅ |</t>
+          <t>|  B,D,F,H  || J |
+| a,c,e,g,i || ∅ |</t>
         </is>
       </c>
       <c r="E41" t="inlineStr">
         <is>
-          <t>0,0041897893</t>
+          <t>0,001448214</t>
         </is>
       </c>
       <c r="F41" t="inlineStr">
         <is>
-          <t>0,025290250778198242</t>
+          <t>0,016705751419067383</t>
         </is>
       </c>
     </row>
@@ -1706,28 +1694,28 @@
       </c>
       <c r="B42" t="inlineStr">
         <is>
-          <t>010101010101010</t>
+          <t>010101010100000</t>
         </is>
       </c>
       <c r="C42" t="inlineStr">
         <is>
-          <t>010101010101010</t>
+          <t>010101010100000</t>
         </is>
       </c>
       <c r="D42" t="inlineStr">
         <is>
-          <t>|  B,D,F,H,J,L  || N |
-| b,d,f,h,j,l,n || ∅ |</t>
+          <t>|  D,F,H,J  || B |
+| b,d,f,h,j || ∅ |</t>
         </is>
       </c>
       <c r="E42" t="inlineStr">
         <is>
-          <t>0,008794069</t>
+          <t>0,0034030676</t>
         </is>
       </c>
       <c r="F42" t="inlineStr">
         <is>
-          <t>0,016762971878051758</t>
+          <t>0,013892889022827148</t>
         </is>
       </c>
     </row>
@@ -1737,28 +1725,28 @@
       </c>
       <c r="B43" t="inlineStr">
         <is>
-          <t>010101010101010</t>
+          <t>010101010100000</t>
         </is>
       </c>
       <c r="C43" t="inlineStr">
         <is>
-          <t>110110110110110</t>
+          <t>110110110100000</t>
         </is>
       </c>
       <c r="D43" t="inlineStr">
         <is>
-          <t>|     B,D,F,H,J,L     || N |
-| a,b,d,e,g,h,j,k,m,n || ∅ |</t>
+          <t>|    B,F,H,J    || D |
+| a,b,d,e,g,h,j || ∅ |</t>
         </is>
       </c>
       <c r="E43" t="inlineStr">
         <is>
-          <t>0,0013378263</t>
+          <t>0,0015337467</t>
         </is>
       </c>
       <c r="F43" t="inlineStr">
         <is>
-          <t>0,08689594268798828</t>
+          <t>0,027936935424804688</t>
         </is>
       </c>
     </row>
@@ -1768,28 +1756,28 @@
       </c>
       <c r="B44" t="inlineStr">
         <is>
-          <t>110110110110110</t>
+          <t>110110110100000</t>
         </is>
       </c>
       <c r="C44" t="inlineStr">
         <is>
-          <t>111111111111111</t>
+          <t>111111111100000</t>
         </is>
       </c>
       <c r="D44" t="inlineStr">
         <is>
-          <t>|     A,B,D,E,G,H,J,K,M,N     || ∅ |
-| b,c,d,e,f,g,h,i,j,k,l,m,n,o || a |</t>
+          <t>|     A,B,D,E,H,J     || G |
+| a,b,c,d,e,f,g,h,i,j || ∅ |</t>
         </is>
       </c>
       <c r="E44" t="inlineStr">
         <is>
-          <t>0,0</t>
+          <t>0,00026786327</t>
         </is>
       </c>
       <c r="F44" t="inlineStr">
         <is>
-          <t>3,844012975692749</t>
+          <t>0,2023019790649414</t>
         </is>
       </c>
     </row>
@@ -1799,28 +1787,28 @@
       </c>
       <c r="B45" t="inlineStr">
         <is>
-          <t>110110110110110</t>
+          <t>110110110100000</t>
         </is>
       </c>
       <c r="C45" t="inlineStr">
         <is>
-          <t>111111111111111</t>
+          <t>111111111000000</t>
         </is>
       </c>
       <c r="D45" t="inlineStr">
         <is>
-          <t>|     A,B,D,E,G,H,J,K,M,N     || ∅ |
-| b,c,d,e,f,g,h,i,j,k,l,m,n,o || a |</t>
+          <t>|    A,B,D,E,G,H    || J |
+| a,b,c,d,e,f,g,h,i || ∅ |</t>
         </is>
       </c>
       <c r="E45" t="inlineStr">
         <is>
-          <t>0,0</t>
+          <t>0,0017379522</t>
         </is>
       </c>
       <c r="F45" t="inlineStr">
         <is>
-          <t>3,8070285320281982</t>
+          <t>0,0972898006439209</t>
         </is>
       </c>
     </row>
@@ -1830,28 +1818,28 @@
       </c>
       <c r="B46" t="inlineStr">
         <is>
-          <t>110110110110110</t>
+          <t>110110110100000</t>
         </is>
       </c>
       <c r="C46" t="inlineStr">
         <is>
-          <t>011111111111111</t>
+          <t>011111111100000</t>
         </is>
       </c>
       <c r="D46" t="inlineStr">
         <is>
-          <t>|    A,B,D,E,G,H,J,K,M,N    || ∅ |
-| c,d,e,f,g,h,i,j,k,l,m,n,o || b |</t>
+          <t>|    A,B,E,G,H,J    || D |
+| b,c,d,e,f,g,h,i,j || ∅ |</t>
         </is>
       </c>
       <c r="E46" t="inlineStr">
         <is>
-          <t>0,0</t>
+          <t>0,0002501011</t>
         </is>
       </c>
       <c r="F46" t="inlineStr">
         <is>
-          <t>1,7314224243164062</t>
+          <t>0,0904240608215332</t>
         </is>
       </c>
     </row>
@@ -1861,28 +1849,28 @@
       </c>
       <c r="B47" t="inlineStr">
         <is>
-          <t>110110110110110</t>
+          <t>110110110100000</t>
         </is>
       </c>
       <c r="C47" t="inlineStr">
         <is>
-          <t>011111111111111</t>
+          <t>011111111000000</t>
         </is>
       </c>
       <c r="D47" t="inlineStr">
         <is>
-          <t>|    A,B,D,E,G,H,J,K,M,N    || ∅ |
-| c,d,e,f,g,h,i,j,k,l,m,n,o || b |</t>
+          <t>|   A,B,D,E,G,H   || J |
+| b,c,d,e,f,g,h,i || ∅ |</t>
         </is>
       </c>
       <c r="E47" t="inlineStr">
         <is>
-          <t>0,0</t>
+          <t>0,0030118823</t>
         </is>
       </c>
       <c r="F47" t="inlineStr">
         <is>
-          <t>1,7736790180206299</t>
+          <t>0,05455136299133301</t>
         </is>
       </c>
     </row>
@@ -1892,28 +1880,28 @@
       </c>
       <c r="B48" t="inlineStr">
         <is>
-          <t>110110110110110</t>
+          <t>110110110100000</t>
         </is>
       </c>
       <c r="C48" t="inlineStr">
         <is>
-          <t>101010101010101</t>
+          <t>101010101000000</t>
         </is>
       </c>
       <c r="D48" t="inlineStr">
         <is>
-          <t>| A,B,D,G,H,J,K,M,N || E |
-|  a,c,e,g,i,k,m,o  || ∅ |</t>
+          <t>| A,B,D,E,G,H || J |
+|  a,c,e,g,i  || ∅ |</t>
         </is>
       </c>
       <c r="E48" t="inlineStr">
         <is>
-          <t>0,0043781996</t>
+          <t>0,001448214</t>
         </is>
       </c>
       <c r="F48" t="inlineStr">
         <is>
-          <t>0,03463029861450195</t>
+          <t>0,022000551223754883</t>
         </is>
       </c>
     </row>
@@ -1923,28 +1911,28 @@
       </c>
       <c r="B49" t="inlineStr">
         <is>
-          <t>110110110110110</t>
+          <t>110110110100000</t>
         </is>
       </c>
       <c r="C49" t="inlineStr">
         <is>
-          <t>010101010101010</t>
+          <t>010101010100000</t>
         </is>
       </c>
       <c r="D49" t="inlineStr">
         <is>
-          <t>| A,B,D,E,H,J,K,M,N || G |
-|   b,d,f,h,j,l,n   || ∅ |</t>
+          <t>| A,B,D,G,H,J || E |
+|  b,d,f,h,j  || ∅ |</t>
         </is>
       </c>
       <c r="E49" t="inlineStr">
         <is>
-          <t>0,0070973635</t>
+          <t>0,0019196868</t>
         </is>
       </c>
       <c r="F49" t="inlineStr">
         <is>
-          <t>0,023804903030395508</t>
+          <t>0,018903017044067383</t>
         </is>
       </c>
     </row>
@@ -1954,28 +1942,28 @@
       </c>
       <c r="B50" t="inlineStr">
         <is>
-          <t>110110110110110</t>
+          <t>110110110100000</t>
         </is>
       </c>
       <c r="C50" t="inlineStr">
         <is>
-          <t>110110110110110</t>
+          <t>110110110100000</t>
         </is>
       </c>
       <c r="D50" t="inlineStr">
         <is>
-          <t>|  A,B,D,E,G,H,J,K,M  || N |
-| a,b,d,e,g,h,j,k,m,n || ∅ |</t>
+          <t>|  B,D,E,G,H,J  || A |
+| a,b,d,e,g,h,j || ∅ |</t>
         </is>
       </c>
       <c r="E50" t="inlineStr">
         <is>
-          <t>0,0013378263</t>
+          <t>0,0013819933</t>
         </is>
       </c>
       <c r="F50" t="inlineStr">
         <is>
-          <t>0,0986027717590332</t>
+          <t>0,03838706016540527</t>
         </is>
       </c>
     </row>
@@ -1985,28 +1973,28 @@
       </c>
       <c r="B51" t="inlineStr">
         <is>
-          <t>101111111111111</t>
+          <t>011111100100000</t>
         </is>
       </c>
       <c r="C51" t="inlineStr">
         <is>
-          <t>101111111111111</t>
+          <t>011111111100000</t>
         </is>
       </c>
       <c r="D51" t="inlineStr">
         <is>
-          <t>| A,C,D,E,F,G,H,I,J,K,L,M,N,O || ∅ |
-|  c,d,e,f,g,h,i,j,k,l,m,n,o  || a |</t>
+          <t>|    B,C,E,F,G,J    || D |
+| b,c,d,e,f,g,h,i,j || ∅ |</t>
         </is>
       </c>
       <c r="E51" t="inlineStr">
         <is>
-          <t>0,0</t>
+          <t>0,0002501011</t>
         </is>
       </c>
       <c r="F51" t="inlineStr">
         <is>
-          <t>2,1886658668518066</t>
+          <t>0,1033632755279541</t>
         </is>
       </c>
     </row>

</xml_diff>